<commit_message>
Update course introduction and publications
</commit_message>
<xml_diff>
--- a/publications.xlsx
+++ b/publications.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mingxunz/Documents/wuwuz.github.io/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F4C006F-A4D9-0A4F-AF4A-5A70519CA60C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2EB8EA-325B-9741-B8ED-7C7C4D67F158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19360" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Publications" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="128">
   <si>
     <t>Year</t>
   </si>
@@ -1345,8 +1345,8 @@
       <c r="A3" t="s">
         <v>91</v>
       </c>
-      <c r="D3" t="s">
-        <v>69</v>
+      <c r="D3">
+        <v>2020</v>
       </c>
       <c r="E3" t="s">
         <v>92</v>

</xml_diff>